<commit_message>
Metadata updated: added info+weight for GPT set
</commit_message>
<xml_diff>
--- a/dataset/metadata.xlsx
+++ b/dataset/metadata.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\fiit\BAKAL\VYSPRO_mini\dataset\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\fiit\BAKAL\VYSPRO_GIT\2026-Podolska-VYSPRO\dataset\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC711887-DC17-47D2-BC93-B004E01CF56E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08F16E39-59AE-4FDF-AB7C-4A4DF2FABCBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{5A607370-1816-435E-9348-DECE98FEA272}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{5A607370-1816-435E-9348-DECE98FEA272}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet3" sheetId="3" r:id="rId2"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId3"/>
+    <sheet name="GPT" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="917" uniqueCount="390">
   <si>
     <t>dish_id</t>
   </si>
@@ -557,6 +558,657 @@
   </si>
   <si>
     <t>fried egg</t>
+  </si>
+  <si>
+    <t>photo_1_2026-04-21_15-21-04.jpg</t>
+  </si>
+  <si>
+    <t>photo_2_2026-04-21_15-21-04.jpg</t>
+  </si>
+  <si>
+    <t>photo_3_2026-04-21_15-21-04.jpg</t>
+  </si>
+  <si>
+    <t>photo_4_2026-04-21_15-21-04.jpg</t>
+  </si>
+  <si>
+    <t>photo_5_2026-04-21_15-21-04.jpg</t>
+  </si>
+  <si>
+    <t>photo_6_2026-04-21_15-21-04.jpg</t>
+  </si>
+  <si>
+    <t>photo_7_2026-04-21_15-21-04.jpg</t>
+  </si>
+  <si>
+    <t>photo_8_2026-04-21_15-21-04.jpg</t>
+  </si>
+  <si>
+    <t>photo_9_2026-04-21_15-21-04.jpg</t>
+  </si>
+  <si>
+    <t>photo_10_2026-04-21_15-21-04.jpg</t>
+  </si>
+  <si>
+    <t>photo_11_2026-04-21_15-21-04.jpg</t>
+  </si>
+  <si>
+    <t>photo_12_2026-04-21_15-21-04.jpg</t>
+  </si>
+  <si>
+    <t>photo_13_2026-04-21_15-21-04.jpg</t>
+  </si>
+  <si>
+    <t>photo_14_2026-04-21_15-21-04.jpg</t>
+  </si>
+  <si>
+    <t>photo_15_2026-04-21_15-21-04.jpg</t>
+  </si>
+  <si>
+    <t>photo_16_2026-04-21_15-21-04.jpg</t>
+  </si>
+  <si>
+    <t>photo_17_2026-04-21_15-21-04.jpg</t>
+  </si>
+  <si>
+    <t>photo_18_2026-04-21_15-21-04.jpg</t>
+  </si>
+  <si>
+    <t>photo_19_2026-04-21_15-21-04.jpg</t>
+  </si>
+  <si>
+    <t>photo_20_2026-04-21_15-21-04.jpg</t>
+  </si>
+  <si>
+    <t>photo_21_2026-04-21_15-21-04.jpg</t>
+  </si>
+  <si>
+    <t>photo_22_2026-04-26_16-48-12.jpg</t>
+  </si>
+  <si>
+    <t>photo_23_2026-04-26_16-48-12.jpg</t>
+  </si>
+  <si>
+    <t>photo_24_2026-04-26_16-48-12.jpg</t>
+  </si>
+  <si>
+    <t>photo_25_2026-04-26_16-48-12.jpg</t>
+  </si>
+  <si>
+    <t>photo_26_2026-04-26_16-48-12.jpg</t>
+  </si>
+  <si>
+    <t>photo_27_2026-04-26_16-48-12.jpg</t>
+  </si>
+  <si>
+    <t>photo_28_2026-04-26_16-48-12.jpg</t>
+  </si>
+  <si>
+    <t>photo_29_2026-04-26_16-48-12.jpg</t>
+  </si>
+  <si>
+    <t>photo_30_2026-04-26_16-48-12.jpg</t>
+  </si>
+  <si>
+    <t>photo_31_2026-04-26_16-48-12.jpg</t>
+  </si>
+  <si>
+    <t>photo_32_2026-04-26_16-48-12.jpg</t>
+  </si>
+  <si>
+    <t>photo_33_2026-04-26_16-48-12.jpg</t>
+  </si>
+  <si>
+    <t>photo_34_2026-04-26_16-48-12.jpg</t>
+  </si>
+  <si>
+    <t>photo_35_2026-04-26_16-48-12.jpg</t>
+  </si>
+  <si>
+    <t>photo_36_2026-04-26_16-48-12.jpg</t>
+  </si>
+  <si>
+    <t>photo_37_2026-04-26_16-48-12.jpg</t>
+  </si>
+  <si>
+    <t>photo_38_2026-04-26_16-48-12.jpg</t>
+  </si>
+  <si>
+    <t>photo_39_2026-04-26_16-48-12.jpg</t>
+  </si>
+  <si>
+    <t>photo_40_2026-04-26_16-48-12.jpg</t>
+  </si>
+  <si>
+    <t>photo_41_2026-04-26_16-48-12.jpg</t>
+  </si>
+  <si>
+    <t>photo_42_2026-04-26_16-48-12.jpg</t>
+  </si>
+  <si>
+    <t>photo_43_2026-04-26_16-48-12.jpg</t>
+  </si>
+  <si>
+    <t>photo_44_2026-04-26_16-48-12.jpg</t>
+  </si>
+  <si>
+    <t>photo_45_2026-04-26_16-48-12.jpg</t>
+  </si>
+  <si>
+    <t>photo_46_2026-04-26_16-48-12.jpg</t>
+  </si>
+  <si>
+    <t>photo_47_2026-04-26_16-48-12.jpg</t>
+  </si>
+  <si>
+    <t>photo_48_2026-04-26_16-48-12.jpg</t>
+  </si>
+  <si>
+    <t>photo_49_2026-04-26_16-48-12.jpg</t>
+  </si>
+  <si>
+    <t>photo_50_2026-04-26_16-48-12.jpg</t>
+  </si>
+  <si>
+    <t>photo_51_2026-04-26_16-48-12.jpg</t>
+  </si>
+  <si>
+    <t>photo_52_2026-04-26_16-48-12.jpg</t>
+  </si>
+  <si>
+    <t>photo_53_2026-04-26_16-48-12.jpg</t>
+  </si>
+  <si>
+    <t>photo_54_2026-04-26_16-48-12.jpg</t>
+  </si>
+  <si>
+    <t>photo_55_2026-04-26_16-48-12.jpg</t>
+  </si>
+  <si>
+    <t>photo_56_2026-04-26_16-48-12.jpg</t>
+  </si>
+  <si>
+    <t>photo_57_2026-04-26_16-48-12.jpg</t>
+  </si>
+  <si>
+    <t>photo_58_2026-04-27_13-42-45.jpg</t>
+  </si>
+  <si>
+    <t>photo_59_2026-04-27_13-42-45.jpg</t>
+  </si>
+  <si>
+    <t>photo_60_2026-04-27_13-42-45.jpg</t>
+  </si>
+  <si>
+    <t>photo_61_2026-04-27_13-42-45.jpg</t>
+  </si>
+  <si>
+    <t>photo_62_2026-04-27_13-42-45.jpg</t>
+  </si>
+  <si>
+    <t>photo_63_2026-04-27_13-42-45.jpg</t>
+  </si>
+  <si>
+    <t>photo_64_2026-04-27_13-42-45.jpg</t>
+  </si>
+  <si>
+    <t>photo_65_2026-04-27_13-42-45.jpg</t>
+  </si>
+  <si>
+    <t>photo_66_2026-04-27_13-42-45.jpg</t>
+  </si>
+  <si>
+    <t>photo_67_2026-04-27_13-42-45.jpg</t>
+  </si>
+  <si>
+    <t>photo_68_2026-04-27_13-42-45.jpg</t>
+  </si>
+  <si>
+    <t>photo_69_2026-04-27_13-42-45.jpg</t>
+  </si>
+  <si>
+    <t>photo_70_2026-04-27_13-42-45.jpg</t>
+  </si>
+  <si>
+    <t>photo_71_2026-04-27_13-42-45.jpg</t>
+  </si>
+  <si>
+    <t>photo_72_2026-04-27_13-42-45.jpg</t>
+  </si>
+  <si>
+    <t>photo_73_2026-04-27_13-42-45.jpg</t>
+  </si>
+  <si>
+    <t>photo_74_2026-04-27_13-42-45.jpg</t>
+  </si>
+  <si>
+    <t>photo_75_2026-04-27_13-42-45.jpg</t>
+  </si>
+  <si>
+    <t>photo_76_2026-04-27_13-42-45.jpg</t>
+  </si>
+  <si>
+    <t>photo_77_2026-04-27_13-42-45.jpg</t>
+  </si>
+  <si>
+    <t>photo_78_2026-04-27_13-42-45.jpg</t>
+  </si>
+  <si>
+    <t>photo_79_2026-04-27_13-42-45.jpg</t>
+  </si>
+  <si>
+    <t>photo_80_2026-04-27_13-42-45.jpg</t>
+  </si>
+  <si>
+    <t>photo_81_2026-04-27_13-42-45.jpg</t>
+  </si>
+  <si>
+    <t>photo_82_2026-04-27_13-42-45.jpg</t>
+  </si>
+  <si>
+    <t>photo_83_2026-04-27_13-42-45.jpg</t>
+  </si>
+  <si>
+    <t>photo_84_2026-04-27_13-42-45.jpg</t>
+  </si>
+  <si>
+    <t>photo_85_2026-04-27_13-42-45.jpg</t>
+  </si>
+  <si>
+    <t>photo_86_2026-04-27_13-42-45.jpg</t>
+  </si>
+  <si>
+    <t>photo_87_2026-04-27_13-42-45.jpg</t>
+  </si>
+  <si>
+    <t>photo_88_2026-04-27_13-42-45.jpg</t>
+  </si>
+  <si>
+    <t>photo_89_2026-04-27_13-42-45.jpg</t>
+  </si>
+  <si>
+    <t>photo_90_2026-04-27_13-42-45.jpg</t>
+  </si>
+  <si>
+    <t>photo_91_2026-04-27_13-42-45.jpg</t>
+  </si>
+  <si>
+    <t>photo_92_2026-04-27_13-42-45.jpg</t>
+  </si>
+  <si>
+    <t>photo_93_2026-04-27_13-42-45.jpg</t>
+  </si>
+  <si>
+    <t>photo_94_2026-04-27_18-09-09.jpg</t>
+  </si>
+  <si>
+    <t>photo_95_2026-04-27_18-09-09.jpg</t>
+  </si>
+  <si>
+    <t>photo_96_2026-04-27_18-09-09.jpg</t>
+  </si>
+  <si>
+    <t>photo_97_2026-04-27_18-09-09.jpg</t>
+  </si>
+  <si>
+    <t>photo_98_2026-04-27_18-09-09.jpg</t>
+  </si>
+  <si>
+    <t>photo_99_2026-04-27_18-09-09.jpg</t>
+  </si>
+  <si>
+    <t>photo_100_2026-04-27_18-09-09.jpg</t>
+  </si>
+  <si>
+    <t>photo_101_2026-04-27_18-09-09.jpg</t>
+  </si>
+  <si>
+    <t>photo_102_2026-04-27_18-09-09.jpg</t>
+  </si>
+  <si>
+    <t>photo_103_2026-04-28_11-03-50.jpg</t>
+  </si>
+  <si>
+    <t>photo_104_2026-04-28_11-03-50.jpg</t>
+  </si>
+  <si>
+    <t>photo_105_2026-04-28_11-03-50.jpg</t>
+  </si>
+  <si>
+    <t>photo_106_2026-04-28_11-03-50.jpg</t>
+  </si>
+  <si>
+    <t>photo_107_2026-04-28_11-03-50.jpg</t>
+  </si>
+  <si>
+    <t>photo_108_2026-04-28_11-03-50.jpg</t>
+  </si>
+  <si>
+    <t>photo_109_2026-04-28_11-03-50.jpg</t>
+  </si>
+  <si>
+    <t>photo_110_2026-04-28_11-03-50.jpg</t>
+  </si>
+  <si>
+    <t>photo_111_2026-04-28_11-03-50.jpg</t>
+  </si>
+  <si>
+    <t>photo_112_2026-04-28_11-03-50.jpg</t>
+  </si>
+  <si>
+    <t>photo_113_2026-04-28_11-03-50.jpg</t>
+  </si>
+  <si>
+    <t>photo_114_2026-04-28_11-03-50.jpg</t>
+  </si>
+  <si>
+    <t>photo_115_2026-04-28_11-03-50.jpg</t>
+  </si>
+  <si>
+    <t>photo_116_2026-04-28_11-03-50.jpg</t>
+  </si>
+  <si>
+    <t>photo_117_2026-04-28_11-03-50.jpg</t>
+  </si>
+  <si>
+    <t>photo_118_2026-04-28_11-03-50.jpg</t>
+  </si>
+  <si>
+    <t>photo_119_2026-04-28_11-03-50.jpg</t>
+  </si>
+  <si>
+    <t>photo_120_2026-04-28_11-03-50.jpg</t>
+  </si>
+  <si>
+    <t>photo_121_2026-04-28_11-03-50.jpg</t>
+  </si>
+  <si>
+    <t>photo_122_2026-04-28_11-03-50.jpg</t>
+  </si>
+  <si>
+    <t>photo_123_2026-04-28_11-03-50.jpg</t>
+  </si>
+  <si>
+    <t>photo_124_2026-04-28_13-43-14.jpg</t>
+  </si>
+  <si>
+    <t>photo_125_2026-04-28_13-43-14.jpg</t>
+  </si>
+  <si>
+    <t>photo_126_2026-04-28_13-43-14.jpg</t>
+  </si>
+  <si>
+    <t>photo_127_2026-04-28_13-43-14.jpg</t>
+  </si>
+  <si>
+    <t>photo_128_2026-04-28_13-43-14.jpg</t>
+  </si>
+  <si>
+    <t>photo_129_2026-04-28_13-43-14.jpg</t>
+  </si>
+  <si>
+    <t>photo_130_2026-04-28_13-43-14.jpg</t>
+  </si>
+  <si>
+    <t>photo_131_2026-04-28_13-43-14.jpg</t>
+  </si>
+  <si>
+    <t>photo_132_2026-04-28_13-43-14.jpg</t>
+  </si>
+  <si>
+    <t>photo_133_2026-04-28_13-43-14.jpg</t>
+  </si>
+  <si>
+    <t>photo_134_2026-04-28_13-43-14.jpg</t>
+  </si>
+  <si>
+    <t>photo_135_2026-04-28_13-43-14.jpg</t>
+  </si>
+  <si>
+    <t>photo_136_2026-04-29_12-20-24.jpg</t>
+  </si>
+  <si>
+    <t>photo_137_2026-04-29_12-20-24.jpg</t>
+  </si>
+  <si>
+    <t>photo_138_2026-04-29_12-20-24.jpg</t>
+  </si>
+  <si>
+    <t>photo_139_2026-04-29_12-20-24.jpg</t>
+  </si>
+  <si>
+    <t>photo_140_2026-04-29_12-20-24.jpg</t>
+  </si>
+  <si>
+    <t>photo_141_2026-04-29_12-20-24.jpg</t>
+  </si>
+  <si>
+    <t>photo_142_2026-04-29_12-20-24.jpg</t>
+  </si>
+  <si>
+    <t>photo_143_2026-04-29_12-20-24.jpg</t>
+  </si>
+  <si>
+    <t>photo_144_2026-04-29_12-20-24.jpg</t>
+  </si>
+  <si>
+    <t>photo_145_2026-04-29_12-20-24.jpg</t>
+  </si>
+  <si>
+    <t>photo_146_2026-04-29_12-20-24.jpg</t>
+  </si>
+  <si>
+    <t>photo_147_2026-04-29_12-20-24.jpg</t>
+  </si>
+  <si>
+    <t>photo_148_2026-04-29_12-20-24.jpg</t>
+  </si>
+  <si>
+    <t>photo_149_2026-04-29_12-20-24.jpg</t>
+  </si>
+  <si>
+    <t>photo_150_2026-04-29_12-20-24.jpg</t>
+  </si>
+  <si>
+    <t>photo_151_2026-04-29_12-20-24.jpg</t>
+  </si>
+  <si>
+    <t>photo_152_2026-04-29_12-20-24.jpg</t>
+  </si>
+  <si>
+    <t>photo_153_2026-04-29_12-20-24.jpg</t>
+  </si>
+  <si>
+    <t>photo_154_2026-04-29_12-20-24.jpg</t>
+  </si>
+  <si>
+    <t>photo_155_2026-04-29_12-20-24.jpg</t>
+  </si>
+  <si>
+    <t>photo_156_2026-04-29_12-20-24.jpg</t>
+  </si>
+  <si>
+    <t>photo_157_2026-04-29_12-20-24.jpg</t>
+  </si>
+  <si>
+    <t>photo_158_2026-04-29_12-20-24.jpg</t>
+  </si>
+  <si>
+    <t>photo_159_2026-04-29_12-20-24.jpg</t>
+  </si>
+  <si>
+    <t>photo_160_2026-04-29_12-20-33.jpg</t>
+  </si>
+  <si>
+    <t>photo_161_2026-04-29_12-20-33.jpg</t>
+  </si>
+  <si>
+    <t>photo_162_2026-04-29_12-20-33.jpg</t>
+  </si>
+  <si>
+    <t>photo_163_2026-04-29_12-20-33.jpg</t>
+  </si>
+  <si>
+    <t>photo_164_2026-04-29_12-20-33.jpg</t>
+  </si>
+  <si>
+    <t>photo_165_2026-04-29_12-20-33.jpg</t>
+  </si>
+  <si>
+    <t>photo name</t>
+  </si>
+  <si>
+    <t>name1</t>
+  </si>
+  <si>
+    <t>weight1</t>
+  </si>
+  <si>
+    <t>name2</t>
+  </si>
+  <si>
+    <t>weight2</t>
+  </si>
+  <si>
+    <t>name3</t>
+  </si>
+  <si>
+    <t>weight3</t>
+  </si>
+  <si>
+    <t>name4</t>
+  </si>
+  <si>
+    <t>weight4</t>
+  </si>
+  <si>
+    <t>Steak</t>
+  </si>
+  <si>
+    <t>Broccoli</t>
+  </si>
+  <si>
+    <t>Potatoes</t>
+  </si>
+  <si>
+    <t>Burger</t>
+  </si>
+  <si>
+    <t>French fries</t>
+  </si>
+  <si>
+    <t>Tomato</t>
+  </si>
+  <si>
+    <t>pizza</t>
+  </si>
+  <si>
+    <t>onion</t>
+  </si>
+  <si>
+    <t>Mushrooms</t>
+  </si>
+  <si>
+    <t>Chicken</t>
+  </si>
+  <si>
+    <t>Salmon</t>
+  </si>
+  <si>
+    <t>Buckwheat</t>
+  </si>
+  <si>
+    <t>Cucumber</t>
+  </si>
+  <si>
+    <t>Sausage</t>
+  </si>
+  <si>
+    <t>potato</t>
+  </si>
+  <si>
+    <t>Carrots</t>
+  </si>
+  <si>
+    <t>Bread</t>
+  </si>
+  <si>
+    <t>Yogurt</t>
+  </si>
+  <si>
+    <t>Apple</t>
+  </si>
+  <si>
+    <t>Cookie</t>
+  </si>
+  <si>
+    <t>Pasta</t>
+  </si>
+  <si>
+    <t>fries</t>
+  </si>
+  <si>
+    <t>Pizza</t>
+  </si>
+  <si>
+    <t>Mozzarella</t>
+  </si>
+  <si>
+    <t>Lettuce</t>
+  </si>
+  <si>
+    <t>Tortilla</t>
+  </si>
+  <si>
+    <t>Fries</t>
+  </si>
+  <si>
+    <t>Rice</t>
+  </si>
+  <si>
+    <t>Beans</t>
+  </si>
+  <si>
+    <t>Potato</t>
+  </si>
+  <si>
+    <t>Onion</t>
+  </si>
+  <si>
+    <t>Carrot</t>
+  </si>
+  <si>
+    <t>Banana</t>
+  </si>
+  <si>
+    <t>Cornie</t>
+  </si>
+  <si>
+    <t>Cheese</t>
+  </si>
+  <si>
+    <t>Egg</t>
+  </si>
+  <si>
+    <t>Mandarin</t>
+  </si>
+  <si>
+    <t>Sushi Philadelphia</t>
+  </si>
+  <si>
+    <t>Soy Sauce</t>
+  </si>
+  <si>
+    <t>Pepper</t>
+  </si>
+  <si>
+    <t>Beetroot</t>
+  </si>
+  <si>
+    <t>Avocado</t>
+  </si>
+  <si>
+    <t>Nuts</t>
   </si>
 </sst>
 </file>
@@ -2366,4 +3018,3967 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D4B05DF-8C29-4B58-8FC1-553488A0031E}">
+  <dimension ref="A1:I166"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="32.5546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>338</v>
+      </c>
+      <c r="B1" t="s">
+        <v>339</v>
+      </c>
+      <c r="C1" t="s">
+        <v>340</v>
+      </c>
+      <c r="D1" t="s">
+        <v>341</v>
+      </c>
+      <c r="E1" t="s">
+        <v>342</v>
+      </c>
+      <c r="F1" t="s">
+        <v>343</v>
+      </c>
+      <c r="G1" t="s">
+        <v>344</v>
+      </c>
+      <c r="H1" t="s">
+        <v>345</v>
+      </c>
+      <c r="I1" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>173</v>
+      </c>
+      <c r="B2" t="s">
+        <v>347</v>
+      </c>
+      <c r="C2">
+        <v>220</v>
+      </c>
+      <c r="D2" t="s">
+        <v>348</v>
+      </c>
+      <c r="E2">
+        <v>130</v>
+      </c>
+      <c r="F2" t="s">
+        <v>349</v>
+      </c>
+      <c r="G2">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>174</v>
+      </c>
+      <c r="B3" t="s">
+        <v>347</v>
+      </c>
+      <c r="C3">
+        <v>220</v>
+      </c>
+      <c r="D3" t="s">
+        <v>348</v>
+      </c>
+      <c r="E3">
+        <v>130</v>
+      </c>
+      <c r="F3" t="s">
+        <v>349</v>
+      </c>
+      <c r="G3">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>175</v>
+      </c>
+      <c r="B4" t="s">
+        <v>347</v>
+      </c>
+      <c r="C4">
+        <v>220</v>
+      </c>
+      <c r="D4" t="s">
+        <v>348</v>
+      </c>
+      <c r="E4">
+        <v>130</v>
+      </c>
+      <c r="F4" t="s">
+        <v>349</v>
+      </c>
+      <c r="G4">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>176</v>
+      </c>
+      <c r="B5" t="s">
+        <v>350</v>
+      </c>
+      <c r="C5">
+        <v>260</v>
+      </c>
+      <c r="D5" t="s">
+        <v>351</v>
+      </c>
+      <c r="E5">
+        <v>150</v>
+      </c>
+      <c r="F5" t="s">
+        <v>352</v>
+      </c>
+      <c r="G5">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>177</v>
+      </c>
+      <c r="B6" t="s">
+        <v>350</v>
+      </c>
+      <c r="C6">
+        <v>260</v>
+      </c>
+      <c r="D6" t="s">
+        <v>351</v>
+      </c>
+      <c r="E6">
+        <v>150</v>
+      </c>
+      <c r="F6" t="s">
+        <v>352</v>
+      </c>
+      <c r="G6">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>178</v>
+      </c>
+      <c r="B7" t="s">
+        <v>350</v>
+      </c>
+      <c r="C7">
+        <v>260</v>
+      </c>
+      <c r="D7" t="s">
+        <v>351</v>
+      </c>
+      <c r="E7">
+        <v>150</v>
+      </c>
+      <c r="F7" t="s">
+        <v>352</v>
+      </c>
+      <c r="G7">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>179</v>
+      </c>
+      <c r="B8" t="s">
+        <v>353</v>
+      </c>
+      <c r="C8">
+        <v>230</v>
+      </c>
+      <c r="D8" t="s">
+        <v>354</v>
+      </c>
+      <c r="E8">
+        <v>55</v>
+      </c>
+      <c r="F8" t="s">
+        <v>355</v>
+      </c>
+      <c r="G8">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>180</v>
+      </c>
+      <c r="B9" t="s">
+        <v>353</v>
+      </c>
+      <c r="C9">
+        <v>230</v>
+      </c>
+      <c r="D9" t="s">
+        <v>354</v>
+      </c>
+      <c r="E9">
+        <v>55</v>
+      </c>
+      <c r="F9" t="s">
+        <v>355</v>
+      </c>
+      <c r="G9">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>181</v>
+      </c>
+      <c r="B10" t="s">
+        <v>353</v>
+      </c>
+      <c r="C10">
+        <v>230</v>
+      </c>
+      <c r="D10" t="s">
+        <v>354</v>
+      </c>
+      <c r="E10">
+        <v>55</v>
+      </c>
+      <c r="F10" t="s">
+        <v>355</v>
+      </c>
+      <c r="G10">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>182</v>
+      </c>
+      <c r="B11" t="s">
+        <v>356</v>
+      </c>
+      <c r="C11">
+        <v>190</v>
+      </c>
+      <c r="D11" t="s">
+        <v>170</v>
+      </c>
+      <c r="E11">
+        <v>180</v>
+      </c>
+      <c r="F11" t="s">
+        <v>348</v>
+      </c>
+      <c r="G11">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>183</v>
+      </c>
+      <c r="B12" t="s">
+        <v>356</v>
+      </c>
+      <c r="C12">
+        <v>190</v>
+      </c>
+      <c r="D12" t="s">
+        <v>170</v>
+      </c>
+      <c r="E12">
+        <v>180</v>
+      </c>
+      <c r="F12" t="s">
+        <v>348</v>
+      </c>
+      <c r="G12">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>184</v>
+      </c>
+      <c r="B13" t="s">
+        <v>356</v>
+      </c>
+      <c r="C13">
+        <v>190</v>
+      </c>
+      <c r="D13" t="s">
+        <v>170</v>
+      </c>
+      <c r="E13">
+        <v>180</v>
+      </c>
+      <c r="F13" t="s">
+        <v>348</v>
+      </c>
+      <c r="G13">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>185</v>
+      </c>
+      <c r="B14" t="s">
+        <v>357</v>
+      </c>
+      <c r="C14">
+        <v>180</v>
+      </c>
+      <c r="D14" t="s">
+        <v>358</v>
+      </c>
+      <c r="E14">
+        <v>170</v>
+      </c>
+      <c r="F14" t="s">
+        <v>359</v>
+      </c>
+      <c r="G14">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>186</v>
+      </c>
+      <c r="B15" t="s">
+        <v>357</v>
+      </c>
+      <c r="C15">
+        <v>180</v>
+      </c>
+      <c r="D15" t="s">
+        <v>358</v>
+      </c>
+      <c r="E15">
+        <v>170</v>
+      </c>
+      <c r="F15" t="s">
+        <v>359</v>
+      </c>
+      <c r="G15">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>187</v>
+      </c>
+      <c r="B16" t="s">
+        <v>357</v>
+      </c>
+      <c r="C16">
+        <v>180</v>
+      </c>
+      <c r="D16" t="s">
+        <v>358</v>
+      </c>
+      <c r="E16">
+        <v>170</v>
+      </c>
+      <c r="F16" t="s">
+        <v>359</v>
+      </c>
+      <c r="G16">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>188</v>
+      </c>
+      <c r="B17" t="s">
+        <v>360</v>
+      </c>
+      <c r="C17">
+        <v>150</v>
+      </c>
+      <c r="D17" t="s">
+        <v>361</v>
+      </c>
+      <c r="E17">
+        <v>190</v>
+      </c>
+      <c r="F17" t="s">
+        <v>362</v>
+      </c>
+      <c r="G17">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>189</v>
+      </c>
+      <c r="B18" t="s">
+        <v>360</v>
+      </c>
+      <c r="C18">
+        <v>150</v>
+      </c>
+      <c r="D18" t="s">
+        <v>361</v>
+      </c>
+      <c r="E18">
+        <v>190</v>
+      </c>
+      <c r="F18" t="s">
+        <v>362</v>
+      </c>
+      <c r="G18">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>190</v>
+      </c>
+      <c r="B19" t="s">
+        <v>360</v>
+      </c>
+      <c r="C19">
+        <v>150</v>
+      </c>
+      <c r="D19" t="s">
+        <v>361</v>
+      </c>
+      <c r="E19">
+        <v>190</v>
+      </c>
+      <c r="F19" t="s">
+        <v>362</v>
+      </c>
+      <c r="G19">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>191</v>
+      </c>
+      <c r="B20" t="s">
+        <v>363</v>
+      </c>
+      <c r="C20">
+        <v>75</v>
+      </c>
+      <c r="D20" t="s">
+        <v>98</v>
+      </c>
+      <c r="E20">
+        <v>55</v>
+      </c>
+      <c r="F20" t="s">
+        <v>364</v>
+      </c>
+      <c r="G20">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>192</v>
+      </c>
+      <c r="B21" t="s">
+        <v>363</v>
+      </c>
+      <c r="C21">
+        <v>75</v>
+      </c>
+      <c r="D21" t="s">
+        <v>98</v>
+      </c>
+      <c r="E21">
+        <v>55</v>
+      </c>
+      <c r="F21" t="s">
+        <v>364</v>
+      </c>
+      <c r="G21">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>193</v>
+      </c>
+      <c r="B22" t="s">
+        <v>363</v>
+      </c>
+      <c r="C22">
+        <v>75</v>
+      </c>
+      <c r="D22" t="s">
+        <v>98</v>
+      </c>
+      <c r="E22">
+        <v>55</v>
+      </c>
+      <c r="F22" t="s">
+        <v>364</v>
+      </c>
+      <c r="G22">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>194</v>
+      </c>
+      <c r="B23" t="s">
+        <v>365</v>
+      </c>
+      <c r="C23">
+        <v>160</v>
+      </c>
+      <c r="D23" t="s">
+        <v>366</v>
+      </c>
+      <c r="E23">
+        <v>45</v>
+      </c>
+      <c r="F23" t="s">
+        <v>95</v>
+      </c>
+      <c r="G23">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>195</v>
+      </c>
+      <c r="B24" t="s">
+        <v>365</v>
+      </c>
+      <c r="C24">
+        <v>160</v>
+      </c>
+      <c r="D24" t="s">
+        <v>366</v>
+      </c>
+      <c r="E24">
+        <v>45</v>
+      </c>
+      <c r="F24" t="s">
+        <v>95</v>
+      </c>
+      <c r="G24">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>196</v>
+      </c>
+      <c r="B25" t="s">
+        <v>365</v>
+      </c>
+      <c r="C25">
+        <v>160</v>
+      </c>
+      <c r="D25" t="s">
+        <v>366</v>
+      </c>
+      <c r="E25">
+        <v>45</v>
+      </c>
+      <c r="F25" t="s">
+        <v>95</v>
+      </c>
+      <c r="G25">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>197</v>
+      </c>
+      <c r="B26" t="s">
+        <v>367</v>
+      </c>
+      <c r="C26">
+        <v>150</v>
+      </c>
+      <c r="D26" t="s">
+        <v>356</v>
+      </c>
+      <c r="E26">
+        <v>150</v>
+      </c>
+      <c r="F26" t="s">
+        <v>352</v>
+      </c>
+      <c r="G26">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>198</v>
+      </c>
+      <c r="B27" t="s">
+        <v>367</v>
+      </c>
+      <c r="C27">
+        <v>150</v>
+      </c>
+      <c r="D27" t="s">
+        <v>356</v>
+      </c>
+      <c r="E27">
+        <v>150</v>
+      </c>
+      <c r="F27" t="s">
+        <v>352</v>
+      </c>
+      <c r="G27">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>199</v>
+      </c>
+      <c r="B28" t="s">
+        <v>367</v>
+      </c>
+      <c r="C28">
+        <v>150</v>
+      </c>
+      <c r="D28" t="s">
+        <v>356</v>
+      </c>
+      <c r="E28">
+        <v>150</v>
+      </c>
+      <c r="F28" t="s">
+        <v>352</v>
+      </c>
+      <c r="G28">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>200</v>
+      </c>
+      <c r="B29" t="s">
+        <v>347</v>
+      </c>
+      <c r="C29">
+        <v>230</v>
+      </c>
+      <c r="D29" t="s">
+        <v>368</v>
+      </c>
+      <c r="E29">
+        <v>140</v>
+      </c>
+      <c r="F29" t="s">
+        <v>354</v>
+      </c>
+      <c r="G29">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>201</v>
+      </c>
+      <c r="B30" t="s">
+        <v>347</v>
+      </c>
+      <c r="C30">
+        <v>230</v>
+      </c>
+      <c r="D30" t="s">
+        <v>368</v>
+      </c>
+      <c r="E30">
+        <v>140</v>
+      </c>
+      <c r="F30" t="s">
+        <v>354</v>
+      </c>
+      <c r="G30">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>202</v>
+      </c>
+      <c r="B31" t="s">
+        <v>347</v>
+      </c>
+      <c r="C31">
+        <v>230</v>
+      </c>
+      <c r="D31" t="s">
+        <v>368</v>
+      </c>
+      <c r="E31">
+        <v>140</v>
+      </c>
+      <c r="F31" t="s">
+        <v>354</v>
+      </c>
+      <c r="G31">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>203</v>
+      </c>
+      <c r="B32" t="s">
+        <v>369</v>
+      </c>
+      <c r="C32">
+        <v>165</v>
+      </c>
+      <c r="D32" t="s">
+        <v>370</v>
+      </c>
+      <c r="E32">
+        <v>70</v>
+      </c>
+      <c r="F32" t="s">
+        <v>352</v>
+      </c>
+      <c r="G32">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>204</v>
+      </c>
+      <c r="B33" t="s">
+        <v>369</v>
+      </c>
+      <c r="C33">
+        <v>165</v>
+      </c>
+      <c r="D33" t="s">
+        <v>370</v>
+      </c>
+      <c r="E33">
+        <v>70</v>
+      </c>
+      <c r="F33" t="s">
+        <v>352</v>
+      </c>
+      <c r="G33">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>205</v>
+      </c>
+      <c r="B34" t="s">
+        <v>369</v>
+      </c>
+      <c r="C34">
+        <v>165</v>
+      </c>
+      <c r="D34" t="s">
+        <v>370</v>
+      </c>
+      <c r="E34">
+        <v>70</v>
+      </c>
+      <c r="F34" t="s">
+        <v>352</v>
+      </c>
+      <c r="G34">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>206</v>
+      </c>
+      <c r="B35" t="s">
+        <v>350</v>
+      </c>
+      <c r="C35">
+        <v>250</v>
+      </c>
+      <c r="D35" t="s">
+        <v>371</v>
+      </c>
+      <c r="E35">
+        <v>35</v>
+      </c>
+      <c r="F35" t="s">
+        <v>359</v>
+      </c>
+      <c r="G35">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>207</v>
+      </c>
+      <c r="B36" t="s">
+        <v>350</v>
+      </c>
+      <c r="C36">
+        <v>250</v>
+      </c>
+      <c r="D36" t="s">
+        <v>371</v>
+      </c>
+      <c r="E36">
+        <v>35</v>
+      </c>
+      <c r="F36" t="s">
+        <v>359</v>
+      </c>
+      <c r="G36">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>208</v>
+      </c>
+      <c r="B37" t="s">
+        <v>350</v>
+      </c>
+      <c r="C37">
+        <v>250</v>
+      </c>
+      <c r="D37" t="s">
+        <v>371</v>
+      </c>
+      <c r="E37">
+        <v>35</v>
+      </c>
+      <c r="F37" t="s">
+        <v>359</v>
+      </c>
+      <c r="G37">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>209</v>
+      </c>
+      <c r="B38" t="s">
+        <v>372</v>
+      </c>
+      <c r="C38">
+        <v>55</v>
+      </c>
+      <c r="D38" t="s">
+        <v>356</v>
+      </c>
+      <c r="E38">
+        <v>150</v>
+      </c>
+      <c r="F38" t="s">
+        <v>352</v>
+      </c>
+      <c r="G38">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>210</v>
+      </c>
+      <c r="B39" t="s">
+        <v>372</v>
+      </c>
+      <c r="C39">
+        <v>55</v>
+      </c>
+      <c r="D39" t="s">
+        <v>356</v>
+      </c>
+      <c r="E39">
+        <v>150</v>
+      </c>
+      <c r="F39" t="s">
+        <v>352</v>
+      </c>
+      <c r="G39">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>211</v>
+      </c>
+      <c r="B40" t="s">
+        <v>372</v>
+      </c>
+      <c r="C40">
+        <v>55</v>
+      </c>
+      <c r="D40" t="s">
+        <v>356</v>
+      </c>
+      <c r="E40">
+        <v>150</v>
+      </c>
+      <c r="F40" t="s">
+        <v>352</v>
+      </c>
+      <c r="G40">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>212</v>
+      </c>
+      <c r="B41" t="s">
+        <v>373</v>
+      </c>
+      <c r="C41">
+        <v>155</v>
+      </c>
+      <c r="D41" t="s">
+        <v>360</v>
+      </c>
+      <c r="E41">
+        <v>130</v>
+      </c>
+      <c r="F41" t="s">
+        <v>352</v>
+      </c>
+      <c r="G41">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>213</v>
+      </c>
+      <c r="B42" t="s">
+        <v>373</v>
+      </c>
+      <c r="C42">
+        <v>155</v>
+      </c>
+      <c r="D42" t="s">
+        <v>360</v>
+      </c>
+      <c r="E42">
+        <v>130</v>
+      </c>
+      <c r="F42" t="s">
+        <v>352</v>
+      </c>
+      <c r="G42">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
+        <v>214</v>
+      </c>
+      <c r="B43" t="s">
+        <v>373</v>
+      </c>
+      <c r="C43">
+        <v>155</v>
+      </c>
+      <c r="D43" t="s">
+        <v>360</v>
+      </c>
+      <c r="E43">
+        <v>130</v>
+      </c>
+      <c r="F43" t="s">
+        <v>352</v>
+      </c>
+      <c r="G43">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
+        <v>215</v>
+      </c>
+      <c r="B44" t="s">
+        <v>374</v>
+      </c>
+      <c r="C44">
+        <v>160</v>
+      </c>
+      <c r="D44" t="s">
+        <v>356</v>
+      </c>
+      <c r="E44">
+        <v>150</v>
+      </c>
+      <c r="F44" t="s">
+        <v>375</v>
+      </c>
+      <c r="G44">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
+        <v>216</v>
+      </c>
+      <c r="B45" t="s">
+        <v>374</v>
+      </c>
+      <c r="C45">
+        <v>160</v>
+      </c>
+      <c r="D45" t="s">
+        <v>356</v>
+      </c>
+      <c r="E45">
+        <v>150</v>
+      </c>
+      <c r="F45" t="s">
+        <v>375</v>
+      </c>
+      <c r="G45">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
+        <v>217</v>
+      </c>
+      <c r="B46" t="s">
+        <v>374</v>
+      </c>
+      <c r="C46">
+        <v>160</v>
+      </c>
+      <c r="D46" t="s">
+        <v>356</v>
+      </c>
+      <c r="E46">
+        <v>150</v>
+      </c>
+      <c r="F46" t="s">
+        <v>375</v>
+      </c>
+      <c r="G46">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>218</v>
+      </c>
+      <c r="B47" t="s">
+        <v>357</v>
+      </c>
+      <c r="C47">
+        <v>180</v>
+      </c>
+      <c r="D47" t="s">
+        <v>376</v>
+      </c>
+      <c r="E47">
+        <v>150</v>
+      </c>
+      <c r="F47" t="s">
+        <v>348</v>
+      </c>
+      <c r="G47">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
+        <v>219</v>
+      </c>
+      <c r="B48" t="s">
+        <v>357</v>
+      </c>
+      <c r="C48">
+        <v>180</v>
+      </c>
+      <c r="D48" t="s">
+        <v>376</v>
+      </c>
+      <c r="E48">
+        <v>150</v>
+      </c>
+      <c r="F48" t="s">
+        <v>348</v>
+      </c>
+      <c r="G48">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>220</v>
+      </c>
+      <c r="B49" t="s">
+        <v>357</v>
+      </c>
+      <c r="C49">
+        <v>180</v>
+      </c>
+      <c r="D49" t="s">
+        <v>376</v>
+      </c>
+      <c r="E49">
+        <v>150</v>
+      </c>
+      <c r="F49" t="s">
+        <v>348</v>
+      </c>
+      <c r="G49">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>221</v>
+      </c>
+      <c r="B50" t="s">
+        <v>367</v>
+      </c>
+      <c r="C50">
+        <v>190</v>
+      </c>
+      <c r="D50" t="s">
+        <v>355</v>
+      </c>
+      <c r="E50">
+        <v>75</v>
+      </c>
+      <c r="F50" t="s">
+        <v>377</v>
+      </c>
+      <c r="G50">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
+        <v>222</v>
+      </c>
+      <c r="B51" t="s">
+        <v>367</v>
+      </c>
+      <c r="C51">
+        <v>190</v>
+      </c>
+      <c r="D51" t="s">
+        <v>355</v>
+      </c>
+      <c r="E51">
+        <v>75</v>
+      </c>
+      <c r="F51" t="s">
+        <v>377</v>
+      </c>
+      <c r="G51">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A52" t="s">
+        <v>223</v>
+      </c>
+      <c r="B52" t="s">
+        <v>367</v>
+      </c>
+      <c r="C52">
+        <v>190</v>
+      </c>
+      <c r="D52" t="s">
+        <v>355</v>
+      </c>
+      <c r="E52">
+        <v>75</v>
+      </c>
+      <c r="F52" t="s">
+        <v>377</v>
+      </c>
+      <c r="G52">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A53" t="s">
+        <v>224</v>
+      </c>
+      <c r="B53" t="s">
+        <v>347</v>
+      </c>
+      <c r="C53">
+        <v>230</v>
+      </c>
+      <c r="D53" t="s">
+        <v>348</v>
+      </c>
+      <c r="E53">
+        <v>115</v>
+      </c>
+      <c r="F53" t="s">
+        <v>378</v>
+      </c>
+      <c r="G53">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A54" t="s">
+        <v>225</v>
+      </c>
+      <c r="B54" t="s">
+        <v>347</v>
+      </c>
+      <c r="C54">
+        <v>230</v>
+      </c>
+      <c r="D54" t="s">
+        <v>348</v>
+      </c>
+      <c r="E54">
+        <v>115</v>
+      </c>
+      <c r="F54" t="s">
+        <v>378</v>
+      </c>
+      <c r="G54">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A55" t="s">
+        <v>226</v>
+      </c>
+      <c r="B55" t="s">
+        <v>347</v>
+      </c>
+      <c r="C55">
+        <v>230</v>
+      </c>
+      <c r="D55" t="s">
+        <v>348</v>
+      </c>
+      <c r="E55">
+        <v>115</v>
+      </c>
+      <c r="F55" t="s">
+        <v>378</v>
+      </c>
+      <c r="G55">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A56" t="s">
+        <v>227</v>
+      </c>
+      <c r="B56" t="s">
+        <v>365</v>
+      </c>
+      <c r="C56">
+        <v>150</v>
+      </c>
+      <c r="D56" t="s">
+        <v>379</v>
+      </c>
+      <c r="E56">
+        <v>120</v>
+      </c>
+      <c r="F56" t="s">
+        <v>364</v>
+      </c>
+      <c r="G56">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A57" t="s">
+        <v>228</v>
+      </c>
+      <c r="B57" t="s">
+        <v>365</v>
+      </c>
+      <c r="C57">
+        <v>150</v>
+      </c>
+      <c r="D57" t="s">
+        <v>379</v>
+      </c>
+      <c r="E57">
+        <v>120</v>
+      </c>
+      <c r="F57" t="s">
+        <v>364</v>
+      </c>
+      <c r="G57">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A58" t="s">
+        <v>229</v>
+      </c>
+      <c r="B58" t="s">
+        <v>365</v>
+      </c>
+      <c r="C58">
+        <v>150</v>
+      </c>
+      <c r="D58" t="s">
+        <v>379</v>
+      </c>
+      <c r="E58">
+        <v>120</v>
+      </c>
+      <c r="F58" t="s">
+        <v>364</v>
+      </c>
+      <c r="G58">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A59" t="s">
+        <v>230</v>
+      </c>
+      <c r="B59" t="s">
+        <v>369</v>
+      </c>
+      <c r="C59">
+        <v>155</v>
+      </c>
+      <c r="D59" t="s">
+        <v>355</v>
+      </c>
+      <c r="E59">
+        <v>85</v>
+      </c>
+      <c r="F59" t="s">
+        <v>377</v>
+      </c>
+      <c r="G59">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A60" t="s">
+        <v>231</v>
+      </c>
+      <c r="B60" t="s">
+        <v>369</v>
+      </c>
+      <c r="C60">
+        <v>155</v>
+      </c>
+      <c r="D60" t="s">
+        <v>355</v>
+      </c>
+      <c r="E60">
+        <v>85</v>
+      </c>
+      <c r="F60" t="s">
+        <v>377</v>
+      </c>
+      <c r="G60">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A61" t="s">
+        <v>232</v>
+      </c>
+      <c r="B61" t="s">
+        <v>369</v>
+      </c>
+      <c r="C61">
+        <v>155</v>
+      </c>
+      <c r="D61" t="s">
+        <v>355</v>
+      </c>
+      <c r="E61">
+        <v>85</v>
+      </c>
+      <c r="F61" t="s">
+        <v>377</v>
+      </c>
+      <c r="G61">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A62" t="s">
+        <v>233</v>
+      </c>
+      <c r="B62" t="s">
+        <v>350</v>
+      </c>
+      <c r="C62">
+        <v>250</v>
+      </c>
+      <c r="D62" t="s">
+        <v>373</v>
+      </c>
+      <c r="E62">
+        <v>135</v>
+      </c>
+      <c r="F62" t="s">
+        <v>371</v>
+      </c>
+      <c r="G62">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A63" t="s">
+        <v>234</v>
+      </c>
+      <c r="B63" t="s">
+        <v>350</v>
+      </c>
+      <c r="C63">
+        <v>250</v>
+      </c>
+      <c r="D63" t="s">
+        <v>373</v>
+      </c>
+      <c r="E63">
+        <v>135</v>
+      </c>
+      <c r="F63" t="s">
+        <v>371</v>
+      </c>
+      <c r="G63">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A64" t="s">
+        <v>235</v>
+      </c>
+      <c r="B64" t="s">
+        <v>350</v>
+      </c>
+      <c r="C64">
+        <v>250</v>
+      </c>
+      <c r="D64" t="s">
+        <v>373</v>
+      </c>
+      <c r="E64">
+        <v>135</v>
+      </c>
+      <c r="F64" t="s">
+        <v>371</v>
+      </c>
+      <c r="G64">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A65" t="s">
+        <v>236</v>
+      </c>
+      <c r="B65" t="s">
+        <v>356</v>
+      </c>
+      <c r="C65">
+        <v>180</v>
+      </c>
+      <c r="D65" t="s">
+        <v>374</v>
+      </c>
+      <c r="E65">
+        <v>210</v>
+      </c>
+      <c r="F65" t="s">
+        <v>380</v>
+      </c>
+      <c r="G65">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A66" t="s">
+        <v>237</v>
+      </c>
+      <c r="B66" t="s">
+        <v>356</v>
+      </c>
+      <c r="C66">
+        <v>180</v>
+      </c>
+      <c r="D66" t="s">
+        <v>374</v>
+      </c>
+      <c r="E66">
+        <v>210</v>
+      </c>
+      <c r="F66" t="s">
+        <v>380</v>
+      </c>
+      <c r="G66">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A67" t="s">
+        <v>238</v>
+      </c>
+      <c r="B67" t="s">
+        <v>356</v>
+      </c>
+      <c r="C67">
+        <v>180</v>
+      </c>
+      <c r="D67" t="s">
+        <v>374</v>
+      </c>
+      <c r="E67">
+        <v>210</v>
+      </c>
+      <c r="F67" t="s">
+        <v>380</v>
+      </c>
+      <c r="G67">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A68" t="s">
+        <v>239</v>
+      </c>
+      <c r="B68" t="s">
+        <v>357</v>
+      </c>
+      <c r="C68">
+        <v>170</v>
+      </c>
+      <c r="D68" t="s">
+        <v>358</v>
+      </c>
+      <c r="E68">
+        <v>180</v>
+      </c>
+      <c r="F68" t="s">
+        <v>375</v>
+      </c>
+      <c r="G68">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A69" t="s">
+        <v>240</v>
+      </c>
+      <c r="B69" t="s">
+        <v>357</v>
+      </c>
+      <c r="C69">
+        <v>170</v>
+      </c>
+      <c r="D69" t="s">
+        <v>358</v>
+      </c>
+      <c r="E69">
+        <v>180</v>
+      </c>
+      <c r="F69" t="s">
+        <v>375</v>
+      </c>
+      <c r="G69">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A70" t="s">
+        <v>241</v>
+      </c>
+      <c r="B70" t="s">
+        <v>357</v>
+      </c>
+      <c r="C70">
+        <v>170</v>
+      </c>
+      <c r="D70" t="s">
+        <v>358</v>
+      </c>
+      <c r="E70">
+        <v>180</v>
+      </c>
+      <c r="F70" t="s">
+        <v>375</v>
+      </c>
+      <c r="G70">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A71" t="s">
+        <v>242</v>
+      </c>
+      <c r="B71" t="s">
+        <v>352</v>
+      </c>
+      <c r="C71">
+        <v>85</v>
+      </c>
+      <c r="D71" t="s">
+        <v>381</v>
+      </c>
+      <c r="E71">
+        <v>70</v>
+      </c>
+      <c r="F71" t="s">
+        <v>363</v>
+      </c>
+      <c r="G71">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="72" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A72" t="s">
+        <v>243</v>
+      </c>
+      <c r="B72" t="s">
+        <v>352</v>
+      </c>
+      <c r="C72">
+        <v>85</v>
+      </c>
+      <c r="D72" t="s">
+        <v>381</v>
+      </c>
+      <c r="E72">
+        <v>70</v>
+      </c>
+      <c r="F72" t="s">
+        <v>363</v>
+      </c>
+      <c r="G72">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="73" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A73" t="s">
+        <v>244</v>
+      </c>
+      <c r="B73" t="s">
+        <v>352</v>
+      </c>
+      <c r="C73">
+        <v>85</v>
+      </c>
+      <c r="D73" t="s">
+        <v>381</v>
+      </c>
+      <c r="E73">
+        <v>70</v>
+      </c>
+      <c r="F73" t="s">
+        <v>363</v>
+      </c>
+      <c r="G73">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="74" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A74" t="s">
+        <v>245</v>
+      </c>
+      <c r="B74" t="s">
+        <v>347</v>
+      </c>
+      <c r="C74">
+        <v>240</v>
+      </c>
+      <c r="D74" t="s">
+        <v>376</v>
+      </c>
+      <c r="E74">
+        <v>190</v>
+      </c>
+      <c r="F74" t="s">
+        <v>377</v>
+      </c>
+      <c r="G74">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="75" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A75" t="s">
+        <v>246</v>
+      </c>
+      <c r="B75" t="s">
+        <v>347</v>
+      </c>
+      <c r="C75">
+        <v>240</v>
+      </c>
+      <c r="D75" t="s">
+        <v>376</v>
+      </c>
+      <c r="E75">
+        <v>190</v>
+      </c>
+      <c r="F75" t="s">
+        <v>377</v>
+      </c>
+      <c r="G75">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="76" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A76" t="s">
+        <v>247</v>
+      </c>
+      <c r="B76" t="s">
+        <v>347</v>
+      </c>
+      <c r="C76">
+        <v>240</v>
+      </c>
+      <c r="D76" t="s">
+        <v>376</v>
+      </c>
+      <c r="E76">
+        <v>190</v>
+      </c>
+      <c r="F76" t="s">
+        <v>377</v>
+      </c>
+      <c r="G76">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="77" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A77" t="s">
+        <v>248</v>
+      </c>
+      <c r="B77" t="s">
+        <v>369</v>
+      </c>
+      <c r="C77">
+        <v>155</v>
+      </c>
+      <c r="D77" t="s">
+        <v>355</v>
+      </c>
+      <c r="E77">
+        <v>85</v>
+      </c>
+      <c r="F77" t="s">
+        <v>377</v>
+      </c>
+      <c r="G77">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="78" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A78" t="s">
+        <v>249</v>
+      </c>
+      <c r="B78" t="s">
+        <v>369</v>
+      </c>
+      <c r="C78">
+        <v>155</v>
+      </c>
+      <c r="D78" t="s">
+        <v>355</v>
+      </c>
+      <c r="E78">
+        <v>85</v>
+      </c>
+      <c r="F78" t="s">
+        <v>377</v>
+      </c>
+      <c r="G78">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="79" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A79" t="s">
+        <v>250</v>
+      </c>
+      <c r="B79" t="s">
+        <v>369</v>
+      </c>
+      <c r="C79">
+        <v>155</v>
+      </c>
+      <c r="D79" t="s">
+        <v>355</v>
+      </c>
+      <c r="E79">
+        <v>85</v>
+      </c>
+      <c r="F79" t="s">
+        <v>377</v>
+      </c>
+      <c r="G79">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="80" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A80" t="s">
+        <v>251</v>
+      </c>
+      <c r="B80" t="s">
+        <v>350</v>
+      </c>
+      <c r="C80">
+        <v>250</v>
+      </c>
+      <c r="D80" t="s">
+        <v>373</v>
+      </c>
+      <c r="E80">
+        <v>135</v>
+      </c>
+      <c r="F80" t="s">
+        <v>371</v>
+      </c>
+      <c r="G80">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="81" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A81" t="s">
+        <v>252</v>
+      </c>
+      <c r="B81" t="s">
+        <v>350</v>
+      </c>
+      <c r="C81">
+        <v>250</v>
+      </c>
+      <c r="D81" t="s">
+        <v>373</v>
+      </c>
+      <c r="E81">
+        <v>135</v>
+      </c>
+      <c r="F81" t="s">
+        <v>371</v>
+      </c>
+      <c r="G81">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="82" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A82" t="s">
+        <v>253</v>
+      </c>
+      <c r="B82" t="s">
+        <v>350</v>
+      </c>
+      <c r="C82">
+        <v>250</v>
+      </c>
+      <c r="D82" t="s">
+        <v>373</v>
+      </c>
+      <c r="E82">
+        <v>135</v>
+      </c>
+      <c r="F82" t="s">
+        <v>371</v>
+      </c>
+      <c r="G82">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="83" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A83" t="s">
+        <v>254</v>
+      </c>
+      <c r="B83" t="s">
+        <v>356</v>
+      </c>
+      <c r="C83">
+        <v>180</v>
+      </c>
+      <c r="D83" t="s">
+        <v>374</v>
+      </c>
+      <c r="E83">
+        <v>210</v>
+      </c>
+      <c r="F83" t="s">
+        <v>380</v>
+      </c>
+      <c r="G83">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="84" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A84" t="s">
+        <v>255</v>
+      </c>
+      <c r="B84" t="s">
+        <v>356</v>
+      </c>
+      <c r="C84">
+        <v>180</v>
+      </c>
+      <c r="D84" t="s">
+        <v>374</v>
+      </c>
+      <c r="E84">
+        <v>210</v>
+      </c>
+      <c r="F84" t="s">
+        <v>380</v>
+      </c>
+      <c r="G84">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="85" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A85" t="s">
+        <v>256</v>
+      </c>
+      <c r="B85" t="s">
+        <v>356</v>
+      </c>
+      <c r="C85">
+        <v>180</v>
+      </c>
+      <c r="D85" t="s">
+        <v>374</v>
+      </c>
+      <c r="E85">
+        <v>210</v>
+      </c>
+      <c r="F85" t="s">
+        <v>380</v>
+      </c>
+      <c r="G85">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="86" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A86" t="s">
+        <v>257</v>
+      </c>
+      <c r="B86" t="s">
+        <v>357</v>
+      </c>
+      <c r="C86">
+        <v>170</v>
+      </c>
+      <c r="D86" t="s">
+        <v>358</v>
+      </c>
+      <c r="E86">
+        <v>180</v>
+      </c>
+      <c r="F86" t="s">
+        <v>375</v>
+      </c>
+      <c r="G86">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="87" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A87" t="s">
+        <v>258</v>
+      </c>
+      <c r="B87" t="s">
+        <v>357</v>
+      </c>
+      <c r="C87">
+        <v>170</v>
+      </c>
+      <c r="D87" t="s">
+        <v>358</v>
+      </c>
+      <c r="E87">
+        <v>180</v>
+      </c>
+      <c r="F87" t="s">
+        <v>375</v>
+      </c>
+      <c r="G87">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="88" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A88" t="s">
+        <v>259</v>
+      </c>
+      <c r="B88" t="s">
+        <v>357</v>
+      </c>
+      <c r="C88">
+        <v>170</v>
+      </c>
+      <c r="D88" t="s">
+        <v>358</v>
+      </c>
+      <c r="E88">
+        <v>180</v>
+      </c>
+      <c r="F88" t="s">
+        <v>375</v>
+      </c>
+      <c r="G88">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="89" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A89" t="s">
+        <v>260</v>
+      </c>
+      <c r="B89" t="s">
+        <v>352</v>
+      </c>
+      <c r="C89">
+        <v>85</v>
+      </c>
+      <c r="D89" t="s">
+        <v>381</v>
+      </c>
+      <c r="E89">
+        <v>70</v>
+      </c>
+      <c r="F89" t="s">
+        <v>363</v>
+      </c>
+      <c r="G89">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="90" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A90" t="s">
+        <v>261</v>
+      </c>
+      <c r="B90" t="s">
+        <v>352</v>
+      </c>
+      <c r="C90">
+        <v>85</v>
+      </c>
+      <c r="D90" t="s">
+        <v>381</v>
+      </c>
+      <c r="E90">
+        <v>70</v>
+      </c>
+      <c r="F90" t="s">
+        <v>363</v>
+      </c>
+      <c r="G90">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="91" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A91" t="s">
+        <v>262</v>
+      </c>
+      <c r="B91" t="s">
+        <v>352</v>
+      </c>
+      <c r="C91">
+        <v>85</v>
+      </c>
+      <c r="D91" t="s">
+        <v>381</v>
+      </c>
+      <c r="E91">
+        <v>70</v>
+      </c>
+      <c r="F91" t="s">
+        <v>363</v>
+      </c>
+      <c r="G91">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="92" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A92" t="s">
+        <v>263</v>
+      </c>
+      <c r="B92" t="s">
+        <v>347</v>
+      </c>
+      <c r="C92">
+        <v>240</v>
+      </c>
+      <c r="D92" t="s">
+        <v>376</v>
+      </c>
+      <c r="E92">
+        <v>190</v>
+      </c>
+      <c r="F92" t="s">
+        <v>377</v>
+      </c>
+      <c r="G92">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="93" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A93" t="s">
+        <v>264</v>
+      </c>
+      <c r="B93" t="s">
+        <v>347</v>
+      </c>
+      <c r="C93">
+        <v>240</v>
+      </c>
+      <c r="D93" t="s">
+        <v>376</v>
+      </c>
+      <c r="E93">
+        <v>190</v>
+      </c>
+      <c r="F93" t="s">
+        <v>377</v>
+      </c>
+      <c r="G93">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="94" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A94" t="s">
+        <v>265</v>
+      </c>
+      <c r="B94" t="s">
+        <v>347</v>
+      </c>
+      <c r="C94">
+        <v>240</v>
+      </c>
+      <c r="D94" t="s">
+        <v>376</v>
+      </c>
+      <c r="E94">
+        <v>190</v>
+      </c>
+      <c r="F94" t="s">
+        <v>377</v>
+      </c>
+      <c r="G94">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="95" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A95" t="s">
+        <v>266</v>
+      </c>
+      <c r="B95" t="s">
+        <v>369</v>
+      </c>
+      <c r="C95">
+        <v>170</v>
+      </c>
+      <c r="D95" t="s">
+        <v>370</v>
+      </c>
+      <c r="E95">
+        <v>75</v>
+      </c>
+      <c r="F95" t="s">
+        <v>348</v>
+      </c>
+      <c r="G95">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="96" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A96" t="s">
+        <v>267</v>
+      </c>
+      <c r="B96" t="s">
+        <v>369</v>
+      </c>
+      <c r="C96">
+        <v>170</v>
+      </c>
+      <c r="D96" t="s">
+        <v>370</v>
+      </c>
+      <c r="E96">
+        <v>75</v>
+      </c>
+      <c r="F96" t="s">
+        <v>348</v>
+      </c>
+      <c r="G96">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="97" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A97" t="s">
+        <v>268</v>
+      </c>
+      <c r="B97" t="s">
+        <v>369</v>
+      </c>
+      <c r="C97">
+        <v>170</v>
+      </c>
+      <c r="D97" t="s">
+        <v>370</v>
+      </c>
+      <c r="E97">
+        <v>75</v>
+      </c>
+      <c r="F97" t="s">
+        <v>348</v>
+      </c>
+      <c r="G97">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="98" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A98" t="s">
+        <v>269</v>
+      </c>
+      <c r="B98" t="s">
+        <v>350</v>
+      </c>
+      <c r="C98">
+        <v>260</v>
+      </c>
+      <c r="D98" t="s">
+        <v>373</v>
+      </c>
+      <c r="E98">
+        <v>150</v>
+      </c>
+      <c r="F98" t="s">
+        <v>352</v>
+      </c>
+      <c r="G98">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="99" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A99" t="s">
+        <v>270</v>
+      </c>
+      <c r="B99" t="s">
+        <v>350</v>
+      </c>
+      <c r="C99">
+        <v>260</v>
+      </c>
+      <c r="D99" t="s">
+        <v>373</v>
+      </c>
+      <c r="E99">
+        <v>150</v>
+      </c>
+      <c r="F99" t="s">
+        <v>352</v>
+      </c>
+      <c r="G99">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="100" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A100" t="s">
+        <v>271</v>
+      </c>
+      <c r="B100" t="s">
+        <v>350</v>
+      </c>
+      <c r="C100">
+        <v>260</v>
+      </c>
+      <c r="D100" t="s">
+        <v>373</v>
+      </c>
+      <c r="E100">
+        <v>150</v>
+      </c>
+      <c r="F100" t="s">
+        <v>352</v>
+      </c>
+      <c r="G100">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="101" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A101" t="s">
+        <v>272</v>
+      </c>
+      <c r="B101" t="s">
+        <v>367</v>
+      </c>
+      <c r="C101">
+        <v>190</v>
+      </c>
+      <c r="D101" t="s">
+        <v>356</v>
+      </c>
+      <c r="E101">
+        <v>160</v>
+      </c>
+      <c r="F101" t="s">
+        <v>355</v>
+      </c>
+      <c r="G101">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="102" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A102" t="s">
+        <v>273</v>
+      </c>
+      <c r="B102" t="s">
+        <v>367</v>
+      </c>
+      <c r="C102">
+        <v>190</v>
+      </c>
+      <c r="D102" t="s">
+        <v>356</v>
+      </c>
+      <c r="E102">
+        <v>160</v>
+      </c>
+      <c r="F102" t="s">
+        <v>355</v>
+      </c>
+      <c r="G102">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="103" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A103" t="s">
+        <v>274</v>
+      </c>
+      <c r="B103" t="s">
+        <v>367</v>
+      </c>
+      <c r="C103">
+        <v>190</v>
+      </c>
+      <c r="D103" t="s">
+        <v>356</v>
+      </c>
+      <c r="E103">
+        <v>160</v>
+      </c>
+      <c r="F103" t="s">
+        <v>355</v>
+      </c>
+      <c r="G103">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="104" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A104" t="s">
+        <v>275</v>
+      </c>
+      <c r="B104" t="s">
+        <v>374</v>
+      </c>
+      <c r="C104">
+        <v>220</v>
+      </c>
+      <c r="D104" t="s">
+        <v>382</v>
+      </c>
+      <c r="E104">
+        <v>95</v>
+      </c>
+      <c r="F104" t="s">
+        <v>359</v>
+      </c>
+      <c r="G104">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="105" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A105" t="s">
+        <v>276</v>
+      </c>
+      <c r="B105" t="s">
+        <v>374</v>
+      </c>
+      <c r="C105">
+        <v>220</v>
+      </c>
+      <c r="D105" t="s">
+        <v>382</v>
+      </c>
+      <c r="E105">
+        <v>95</v>
+      </c>
+      <c r="F105" t="s">
+        <v>359</v>
+      </c>
+      <c r="G105">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="106" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A106" t="s">
+        <v>277</v>
+      </c>
+      <c r="B106" t="s">
+        <v>374</v>
+      </c>
+      <c r="C106">
+        <v>220</v>
+      </c>
+      <c r="D106" t="s">
+        <v>382</v>
+      </c>
+      <c r="E106">
+        <v>95</v>
+      </c>
+      <c r="F106" t="s">
+        <v>359</v>
+      </c>
+      <c r="G106">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="107" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A107" t="s">
+        <v>278</v>
+      </c>
+      <c r="B107" t="s">
+        <v>357</v>
+      </c>
+      <c r="C107">
+        <v>180</v>
+      </c>
+      <c r="D107" t="s">
+        <v>376</v>
+      </c>
+      <c r="E107">
+        <v>170</v>
+      </c>
+      <c r="F107" t="s">
+        <v>348</v>
+      </c>
+      <c r="G107">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="108" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A108" t="s">
+        <v>279</v>
+      </c>
+      <c r="B108" t="s">
+        <v>357</v>
+      </c>
+      <c r="C108">
+        <v>180</v>
+      </c>
+      <c r="D108" t="s">
+        <v>376</v>
+      </c>
+      <c r="E108">
+        <v>170</v>
+      </c>
+      <c r="F108" t="s">
+        <v>348</v>
+      </c>
+      <c r="G108">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="109" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A109" t="s">
+        <v>280</v>
+      </c>
+      <c r="B109" t="s">
+        <v>357</v>
+      </c>
+      <c r="C109">
+        <v>180</v>
+      </c>
+      <c r="D109" t="s">
+        <v>376</v>
+      </c>
+      <c r="E109">
+        <v>170</v>
+      </c>
+      <c r="F109" t="s">
+        <v>348</v>
+      </c>
+      <c r="G109">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="110" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A110" t="s">
+        <v>281</v>
+      </c>
+      <c r="B110" t="s">
+        <v>347</v>
+      </c>
+      <c r="C110">
+        <v>250</v>
+      </c>
+      <c r="D110" t="s">
+        <v>375</v>
+      </c>
+      <c r="E110">
+        <v>120</v>
+      </c>
+      <c r="F110" t="s">
+        <v>378</v>
+      </c>
+      <c r="G110">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="111" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A111" t="s">
+        <v>282</v>
+      </c>
+      <c r="B111" t="s">
+        <v>347</v>
+      </c>
+      <c r="C111">
+        <v>250</v>
+      </c>
+      <c r="D111" t="s">
+        <v>375</v>
+      </c>
+      <c r="E111">
+        <v>120</v>
+      </c>
+      <c r="F111" t="s">
+        <v>378</v>
+      </c>
+      <c r="G111">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="112" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A112" t="s">
+        <v>283</v>
+      </c>
+      <c r="B112" t="s">
+        <v>347</v>
+      </c>
+      <c r="C112">
+        <v>250</v>
+      </c>
+      <c r="D112" t="s">
+        <v>375</v>
+      </c>
+      <c r="E112">
+        <v>120</v>
+      </c>
+      <c r="F112" t="s">
+        <v>378</v>
+      </c>
+      <c r="G112">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="113" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A113" t="s">
+        <v>284</v>
+      </c>
+      <c r="B113" t="s">
+        <v>369</v>
+      </c>
+      <c r="C113">
+        <v>165</v>
+      </c>
+      <c r="D113" t="s">
+        <v>377</v>
+      </c>
+      <c r="E113">
+        <v>45</v>
+      </c>
+      <c r="F113" t="s">
+        <v>352</v>
+      </c>
+      <c r="G113">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="114" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A114" t="s">
+        <v>285</v>
+      </c>
+      <c r="B114" t="s">
+        <v>369</v>
+      </c>
+      <c r="C114">
+        <v>165</v>
+      </c>
+      <c r="D114" t="s">
+        <v>377</v>
+      </c>
+      <c r="E114">
+        <v>45</v>
+      </c>
+      <c r="F114" t="s">
+        <v>352</v>
+      </c>
+      <c r="G114">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="115" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A115" t="s">
+        <v>286</v>
+      </c>
+      <c r="B115" t="s">
+        <v>369</v>
+      </c>
+      <c r="C115">
+        <v>165</v>
+      </c>
+      <c r="D115" t="s">
+        <v>377</v>
+      </c>
+      <c r="E115">
+        <v>45</v>
+      </c>
+      <c r="F115" t="s">
+        <v>352</v>
+      </c>
+      <c r="G115">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="116" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A116" t="s">
+        <v>287</v>
+      </c>
+      <c r="B116" t="s">
+        <v>350</v>
+      </c>
+      <c r="C116">
+        <v>260</v>
+      </c>
+      <c r="D116" t="s">
+        <v>373</v>
+      </c>
+      <c r="E116">
+        <v>155</v>
+      </c>
+      <c r="F116" t="s">
+        <v>359</v>
+      </c>
+      <c r="G116">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="117" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A117" t="s">
+        <v>288</v>
+      </c>
+      <c r="B117" t="s">
+        <v>350</v>
+      </c>
+      <c r="C117">
+        <v>260</v>
+      </c>
+      <c r="D117" t="s">
+        <v>373</v>
+      </c>
+      <c r="E117">
+        <v>155</v>
+      </c>
+      <c r="F117" t="s">
+        <v>359</v>
+      </c>
+      <c r="G117">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="118" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A118" t="s">
+        <v>289</v>
+      </c>
+      <c r="B118" t="s">
+        <v>350</v>
+      </c>
+      <c r="C118">
+        <v>260</v>
+      </c>
+      <c r="D118" t="s">
+        <v>373</v>
+      </c>
+      <c r="E118">
+        <v>155</v>
+      </c>
+      <c r="F118" t="s">
+        <v>359</v>
+      </c>
+      <c r="G118">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="119" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A119" t="s">
+        <v>290</v>
+      </c>
+      <c r="B119" t="s">
+        <v>356</v>
+      </c>
+      <c r="C119">
+        <v>170</v>
+      </c>
+      <c r="D119" t="s">
+        <v>374</v>
+      </c>
+      <c r="E119">
+        <v>180</v>
+      </c>
+      <c r="F119" t="s">
+        <v>348</v>
+      </c>
+      <c r="G119">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="120" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A120" t="s">
+        <v>291</v>
+      </c>
+      <c r="B120" t="s">
+        <v>356</v>
+      </c>
+      <c r="C120">
+        <v>170</v>
+      </c>
+      <c r="D120" t="s">
+        <v>374</v>
+      </c>
+      <c r="E120">
+        <v>180</v>
+      </c>
+      <c r="F120" t="s">
+        <v>348</v>
+      </c>
+      <c r="G120">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="121" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A121" t="s">
+        <v>292</v>
+      </c>
+      <c r="B121" t="s">
+        <v>356</v>
+      </c>
+      <c r="C121">
+        <v>170</v>
+      </c>
+      <c r="D121" t="s">
+        <v>374</v>
+      </c>
+      <c r="E121">
+        <v>180</v>
+      </c>
+      <c r="F121" t="s">
+        <v>348</v>
+      </c>
+      <c r="G121">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="122" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A122" t="s">
+        <v>293</v>
+      </c>
+      <c r="B122" t="s">
+        <v>367</v>
+      </c>
+      <c r="C122">
+        <v>210</v>
+      </c>
+      <c r="D122" t="s">
+        <v>370</v>
+      </c>
+      <c r="E122">
+        <v>80</v>
+      </c>
+      <c r="F122" t="s">
+        <v>352</v>
+      </c>
+      <c r="G122">
+        <v>95</v>
+      </c>
+      <c r="H122" t="s">
+        <v>348</v>
+      </c>
+      <c r="I122">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="123" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A123" t="s">
+        <v>294</v>
+      </c>
+      <c r="B123" t="s">
+        <v>367</v>
+      </c>
+      <c r="C123">
+        <v>210</v>
+      </c>
+      <c r="D123" t="s">
+        <v>370</v>
+      </c>
+      <c r="E123">
+        <v>80</v>
+      </c>
+      <c r="F123" t="s">
+        <v>352</v>
+      </c>
+      <c r="G123">
+        <v>95</v>
+      </c>
+      <c r="H123" t="s">
+        <v>348</v>
+      </c>
+      <c r="I123">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="124" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A124" t="s">
+        <v>295</v>
+      </c>
+      <c r="B124" t="s">
+        <v>367</v>
+      </c>
+      <c r="C124">
+        <v>210</v>
+      </c>
+      <c r="D124" t="s">
+        <v>370</v>
+      </c>
+      <c r="E124">
+        <v>80</v>
+      </c>
+      <c r="F124" t="s">
+        <v>352</v>
+      </c>
+      <c r="G124">
+        <v>95</v>
+      </c>
+      <c r="H124" t="s">
+        <v>348</v>
+      </c>
+      <c r="I124">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="125" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A125" t="s">
+        <v>296</v>
+      </c>
+      <c r="B125" t="s">
+        <v>363</v>
+      </c>
+      <c r="C125">
+        <v>55</v>
+      </c>
+      <c r="D125" t="s">
+        <v>360</v>
+      </c>
+      <c r="E125">
+        <v>130</v>
+      </c>
+      <c r="F125" t="s">
+        <v>381</v>
+      </c>
+      <c r="G125">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="126" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A126" t="s">
+        <v>297</v>
+      </c>
+      <c r="B126" t="s">
+        <v>363</v>
+      </c>
+      <c r="C126">
+        <v>55</v>
+      </c>
+      <c r="D126" t="s">
+        <v>360</v>
+      </c>
+      <c r="E126">
+        <v>130</v>
+      </c>
+      <c r="F126" t="s">
+        <v>381</v>
+      </c>
+      <c r="G126">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="127" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A127" t="s">
+        <v>298</v>
+      </c>
+      <c r="B127" t="s">
+        <v>363</v>
+      </c>
+      <c r="C127">
+        <v>55</v>
+      </c>
+      <c r="D127" t="s">
+        <v>360</v>
+      </c>
+      <c r="E127">
+        <v>130</v>
+      </c>
+      <c r="F127" t="s">
+        <v>381</v>
+      </c>
+      <c r="G127">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="128" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A128" t="s">
+        <v>299</v>
+      </c>
+      <c r="B128" t="s">
+        <v>357</v>
+      </c>
+      <c r="C128">
+        <v>180</v>
+      </c>
+      <c r="D128" t="s">
+        <v>358</v>
+      </c>
+      <c r="E128">
+        <v>190</v>
+      </c>
+      <c r="F128" t="s">
+        <v>377</v>
+      </c>
+      <c r="G128">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="129" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A129" t="s">
+        <v>300</v>
+      </c>
+      <c r="B129" t="s">
+        <v>357</v>
+      </c>
+      <c r="C129">
+        <v>180</v>
+      </c>
+      <c r="D129" t="s">
+        <v>358</v>
+      </c>
+      <c r="E129">
+        <v>190</v>
+      </c>
+      <c r="F129" t="s">
+        <v>377</v>
+      </c>
+      <c r="G129">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="130" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A130" t="s">
+        <v>301</v>
+      </c>
+      <c r="B130" t="s">
+        <v>357</v>
+      </c>
+      <c r="C130">
+        <v>180</v>
+      </c>
+      <c r="D130" t="s">
+        <v>358</v>
+      </c>
+      <c r="E130">
+        <v>190</v>
+      </c>
+      <c r="F130" t="s">
+        <v>377</v>
+      </c>
+      <c r="G130">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="131" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A131" t="s">
+        <v>302</v>
+      </c>
+      <c r="B131" t="s">
+        <v>347</v>
+      </c>
+      <c r="C131">
+        <v>210</v>
+      </c>
+      <c r="D131" t="s">
+        <v>376</v>
+      </c>
+      <c r="E131">
+        <v>180</v>
+      </c>
+      <c r="F131" t="s">
+        <v>348</v>
+      </c>
+      <c r="G131">
+        <v>120</v>
+      </c>
+      <c r="H131" t="s">
+        <v>377</v>
+      </c>
+      <c r="I131">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="132" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A132" t="s">
+        <v>303</v>
+      </c>
+      <c r="B132" t="s">
+        <v>347</v>
+      </c>
+      <c r="C132">
+        <v>210</v>
+      </c>
+      <c r="D132" t="s">
+        <v>376</v>
+      </c>
+      <c r="E132">
+        <v>180</v>
+      </c>
+      <c r="F132" t="s">
+        <v>348</v>
+      </c>
+      <c r="G132">
+        <v>120</v>
+      </c>
+      <c r="H132" t="s">
+        <v>377</v>
+      </c>
+      <c r="I132">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="133" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A133" t="s">
+        <v>304</v>
+      </c>
+      <c r="B133" t="s">
+        <v>347</v>
+      </c>
+      <c r="C133">
+        <v>210</v>
+      </c>
+      <c r="D133" t="s">
+        <v>376</v>
+      </c>
+      <c r="E133">
+        <v>180</v>
+      </c>
+      <c r="F133" t="s">
+        <v>348</v>
+      </c>
+      <c r="G133">
+        <v>120</v>
+      </c>
+      <c r="H133" t="s">
+        <v>377</v>
+      </c>
+      <c r="I133">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="134" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A134" t="s">
+        <v>305</v>
+      </c>
+      <c r="B134" t="s">
+        <v>365</v>
+      </c>
+      <c r="C134">
+        <v>150</v>
+      </c>
+      <c r="D134" t="s">
+        <v>383</v>
+      </c>
+      <c r="E134">
+        <v>120</v>
+      </c>
+      <c r="F134" t="s">
+        <v>366</v>
+      </c>
+      <c r="G134">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="135" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A135" t="s">
+        <v>306</v>
+      </c>
+      <c r="B135" t="s">
+        <v>365</v>
+      </c>
+      <c r="C135">
+        <v>150</v>
+      </c>
+      <c r="D135" t="s">
+        <v>383</v>
+      </c>
+      <c r="E135">
+        <v>120</v>
+      </c>
+      <c r="F135" t="s">
+        <v>366</v>
+      </c>
+      <c r="G135">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="136" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A136" t="s">
+        <v>307</v>
+      </c>
+      <c r="B136" t="s">
+        <v>365</v>
+      </c>
+      <c r="C136">
+        <v>150</v>
+      </c>
+      <c r="D136" t="s">
+        <v>383</v>
+      </c>
+      <c r="E136">
+        <v>120</v>
+      </c>
+      <c r="F136" t="s">
+        <v>366</v>
+      </c>
+      <c r="G136">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="137" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A137" t="s">
+        <v>308</v>
+      </c>
+      <c r="B137" t="s">
+        <v>357</v>
+      </c>
+      <c r="C137">
+        <v>200</v>
+      </c>
+      <c r="D137" t="s">
+        <v>376</v>
+      </c>
+      <c r="E137">
+        <v>180</v>
+      </c>
+      <c r="F137" t="s">
+        <v>348</v>
+      </c>
+      <c r="G137">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="138" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A138" t="s">
+        <v>309</v>
+      </c>
+      <c r="B138" t="s">
+        <v>357</v>
+      </c>
+      <c r="C138">
+        <v>200</v>
+      </c>
+      <c r="D138" t="s">
+        <v>376</v>
+      </c>
+      <c r="E138">
+        <v>180</v>
+      </c>
+      <c r="F138" t="s">
+        <v>348</v>
+      </c>
+      <c r="G138">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="139" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A139" t="s">
+        <v>310</v>
+      </c>
+      <c r="B139" t="s">
+        <v>357</v>
+      </c>
+      <c r="C139">
+        <v>200</v>
+      </c>
+      <c r="D139" t="s">
+        <v>376</v>
+      </c>
+      <c r="E139">
+        <v>180</v>
+      </c>
+      <c r="F139" t="s">
+        <v>348</v>
+      </c>
+      <c r="G139">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="140" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A140" t="s">
+        <v>311</v>
+      </c>
+      <c r="B140" t="s">
+        <v>357</v>
+      </c>
+      <c r="C140">
+        <v>180</v>
+      </c>
+      <c r="D140" t="s">
+        <v>374</v>
+      </c>
+      <c r="E140">
+        <v>200</v>
+      </c>
+      <c r="F140" t="s">
+        <v>375</v>
+      </c>
+      <c r="G140">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="141" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A141" t="s">
+        <v>312</v>
+      </c>
+      <c r="B141" t="s">
+        <v>357</v>
+      </c>
+      <c r="C141">
+        <v>180</v>
+      </c>
+      <c r="D141" t="s">
+        <v>374</v>
+      </c>
+      <c r="E141">
+        <v>200</v>
+      </c>
+      <c r="F141" t="s">
+        <v>375</v>
+      </c>
+      <c r="G141">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="142" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A142" t="s">
+        <v>313</v>
+      </c>
+      <c r="B142" t="s">
+        <v>357</v>
+      </c>
+      <c r="C142">
+        <v>180</v>
+      </c>
+      <c r="D142" t="s">
+        <v>374</v>
+      </c>
+      <c r="E142">
+        <v>200</v>
+      </c>
+      <c r="F142" t="s">
+        <v>375</v>
+      </c>
+      <c r="G142">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="143" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A143" t="s">
+        <v>314</v>
+      </c>
+      <c r="B143" t="s">
+        <v>369</v>
+      </c>
+      <c r="C143">
+        <v>190</v>
+      </c>
+      <c r="D143" t="s">
+        <v>370</v>
+      </c>
+      <c r="E143">
+        <v>80</v>
+      </c>
+      <c r="F143" t="s">
+        <v>382</v>
+      </c>
+      <c r="G143">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="144" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A144" t="s">
+        <v>315</v>
+      </c>
+      <c r="B144" t="s">
+        <v>369</v>
+      </c>
+      <c r="C144">
+        <v>190</v>
+      </c>
+      <c r="D144" t="s">
+        <v>370</v>
+      </c>
+      <c r="E144">
+        <v>80</v>
+      </c>
+      <c r="F144" t="s">
+        <v>382</v>
+      </c>
+      <c r="G144">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="145" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A145" t="s">
+        <v>316</v>
+      </c>
+      <c r="B145" t="s">
+        <v>369</v>
+      </c>
+      <c r="C145">
+        <v>190</v>
+      </c>
+      <c r="D145" t="s">
+        <v>370</v>
+      </c>
+      <c r="E145">
+        <v>80</v>
+      </c>
+      <c r="F145" t="s">
+        <v>382</v>
+      </c>
+      <c r="G145">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="146" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A146" t="s">
+        <v>317</v>
+      </c>
+      <c r="B146" t="s">
+        <v>384</v>
+      </c>
+      <c r="C146">
+        <v>180</v>
+      </c>
+      <c r="D146" t="s">
+        <v>385</v>
+      </c>
+      <c r="E146">
+        <v>35</v>
+      </c>
+      <c r="F146" t="s">
+        <v>386</v>
+      </c>
+      <c r="G146">
+        <v>90</v>
+      </c>
+      <c r="H146" t="s">
+        <v>387</v>
+      </c>
+      <c r="I146">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="147" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A147" t="s">
+        <v>318</v>
+      </c>
+      <c r="B147" t="s">
+        <v>384</v>
+      </c>
+      <c r="C147">
+        <v>180</v>
+      </c>
+      <c r="D147" t="s">
+        <v>385</v>
+      </c>
+      <c r="E147">
+        <v>35</v>
+      </c>
+      <c r="F147" t="s">
+        <v>386</v>
+      </c>
+      <c r="G147">
+        <v>90</v>
+      </c>
+      <c r="H147" t="s">
+        <v>387</v>
+      </c>
+      <c r="I147">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="148" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A148" t="s">
+        <v>319</v>
+      </c>
+      <c r="B148" t="s">
+        <v>384</v>
+      </c>
+      <c r="C148">
+        <v>180</v>
+      </c>
+      <c r="D148" t="s">
+        <v>385</v>
+      </c>
+      <c r="E148">
+        <v>35</v>
+      </c>
+      <c r="F148" t="s">
+        <v>386</v>
+      </c>
+      <c r="G148">
+        <v>90</v>
+      </c>
+      <c r="H148" t="s">
+        <v>387</v>
+      </c>
+      <c r="I148">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="149" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A149" t="s">
+        <v>320</v>
+      </c>
+      <c r="B149" t="s">
+        <v>384</v>
+      </c>
+      <c r="C149">
+        <v>120</v>
+      </c>
+      <c r="D149" t="s">
+        <v>388</v>
+      </c>
+      <c r="E149">
+        <v>110</v>
+      </c>
+      <c r="F149" t="s">
+        <v>389</v>
+      </c>
+      <c r="G149">
+        <v>45</v>
+      </c>
+      <c r="H149" t="s">
+        <v>385</v>
+      </c>
+      <c r="I149">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="150" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A150" t="s">
+        <v>321</v>
+      </c>
+      <c r="B150" t="s">
+        <v>384</v>
+      </c>
+      <c r="C150">
+        <v>120</v>
+      </c>
+      <c r="D150" t="s">
+        <v>388</v>
+      </c>
+      <c r="E150">
+        <v>110</v>
+      </c>
+      <c r="F150" t="s">
+        <v>389</v>
+      </c>
+      <c r="G150">
+        <v>45</v>
+      </c>
+      <c r="H150" t="s">
+        <v>385</v>
+      </c>
+      <c r="I150">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="151" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A151" t="s">
+        <v>322</v>
+      </c>
+      <c r="B151" t="s">
+        <v>384</v>
+      </c>
+      <c r="C151">
+        <v>120</v>
+      </c>
+      <c r="D151" t="s">
+        <v>388</v>
+      </c>
+      <c r="E151">
+        <v>110</v>
+      </c>
+      <c r="F151" t="s">
+        <v>389</v>
+      </c>
+      <c r="G151">
+        <v>45</v>
+      </c>
+      <c r="H151" t="s">
+        <v>385</v>
+      </c>
+      <c r="I151">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="152" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A152" t="s">
+        <v>323</v>
+      </c>
+      <c r="B152" t="s">
+        <v>388</v>
+      </c>
+      <c r="C152">
+        <v>130</v>
+      </c>
+      <c r="D152" t="s">
+        <v>386</v>
+      </c>
+      <c r="E152">
+        <v>95</v>
+      </c>
+      <c r="F152" t="s">
+        <v>389</v>
+      </c>
+      <c r="G152">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="153" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A153" t="s">
+        <v>324</v>
+      </c>
+      <c r="B153" t="s">
+        <v>388</v>
+      </c>
+      <c r="C153">
+        <v>130</v>
+      </c>
+      <c r="D153" t="s">
+        <v>386</v>
+      </c>
+      <c r="E153">
+        <v>95</v>
+      </c>
+      <c r="F153" t="s">
+        <v>389</v>
+      </c>
+      <c r="G153">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="154" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A154" t="s">
+        <v>325</v>
+      </c>
+      <c r="B154" t="s">
+        <v>388</v>
+      </c>
+      <c r="C154">
+        <v>130</v>
+      </c>
+      <c r="D154" t="s">
+        <v>386</v>
+      </c>
+      <c r="E154">
+        <v>95</v>
+      </c>
+      <c r="F154" t="s">
+        <v>389</v>
+      </c>
+      <c r="G154">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="155" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A155" t="s">
+        <v>326</v>
+      </c>
+      <c r="B155" t="s">
+        <v>384</v>
+      </c>
+      <c r="C155">
+        <v>120</v>
+      </c>
+      <c r="D155" t="s">
+        <v>387</v>
+      </c>
+      <c r="E155">
+        <v>170</v>
+      </c>
+      <c r="F155" t="s">
+        <v>389</v>
+      </c>
+      <c r="G155">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="156" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A156" t="s">
+        <v>327</v>
+      </c>
+      <c r="B156" t="s">
+        <v>384</v>
+      </c>
+      <c r="C156">
+        <v>120</v>
+      </c>
+      <c r="D156" t="s">
+        <v>387</v>
+      </c>
+      <c r="E156">
+        <v>170</v>
+      </c>
+      <c r="F156" t="s">
+        <v>389</v>
+      </c>
+      <c r="G156">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="157" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A157" t="s">
+        <v>328</v>
+      </c>
+      <c r="B157" t="s">
+        <v>384</v>
+      </c>
+      <c r="C157">
+        <v>120</v>
+      </c>
+      <c r="D157" t="s">
+        <v>387</v>
+      </c>
+      <c r="E157">
+        <v>170</v>
+      </c>
+      <c r="F157" t="s">
+        <v>389</v>
+      </c>
+      <c r="G157">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="158" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A158" t="s">
+        <v>329</v>
+      </c>
+      <c r="B158" t="s">
+        <v>386</v>
+      </c>
+      <c r="C158">
+        <v>95</v>
+      </c>
+      <c r="D158" t="s">
+        <v>387</v>
+      </c>
+      <c r="E158">
+        <v>160</v>
+      </c>
+      <c r="F158" t="s">
+        <v>388</v>
+      </c>
+      <c r="G158">
+        <v>130</v>
+      </c>
+      <c r="H158" t="s">
+        <v>385</v>
+      </c>
+      <c r="I158">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="159" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A159" t="s">
+        <v>330</v>
+      </c>
+      <c r="B159" t="s">
+        <v>386</v>
+      </c>
+      <c r="C159">
+        <v>95</v>
+      </c>
+      <c r="D159" t="s">
+        <v>387</v>
+      </c>
+      <c r="E159">
+        <v>160</v>
+      </c>
+      <c r="F159" t="s">
+        <v>388</v>
+      </c>
+      <c r="G159">
+        <v>130</v>
+      </c>
+      <c r="H159" t="s">
+        <v>385</v>
+      </c>
+      <c r="I159">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="160" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A160" t="s">
+        <v>331</v>
+      </c>
+      <c r="B160" t="s">
+        <v>386</v>
+      </c>
+      <c r="C160">
+        <v>95</v>
+      </c>
+      <c r="D160" t="s">
+        <v>387</v>
+      </c>
+      <c r="E160">
+        <v>160</v>
+      </c>
+      <c r="F160" t="s">
+        <v>388</v>
+      </c>
+      <c r="G160">
+        <v>130</v>
+      </c>
+      <c r="H160" t="s">
+        <v>385</v>
+      </c>
+      <c r="I160">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="161" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A161" t="s">
+        <v>332</v>
+      </c>
+      <c r="B161" t="s">
+        <v>386</v>
+      </c>
+      <c r="C161">
+        <v>150</v>
+      </c>
+      <c r="D161" t="s">
+        <v>387</v>
+      </c>
+      <c r="E161">
+        <v>120</v>
+      </c>
+      <c r="F161" t="s">
+        <v>388</v>
+      </c>
+      <c r="G161">
+        <v>85</v>
+      </c>
+      <c r="H161" t="s">
+        <v>385</v>
+      </c>
+      <c r="I161">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="162" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A162" t="s">
+        <v>333</v>
+      </c>
+      <c r="B162" t="s">
+        <v>386</v>
+      </c>
+      <c r="C162">
+        <v>150</v>
+      </c>
+      <c r="D162" t="s">
+        <v>387</v>
+      </c>
+      <c r="E162">
+        <v>120</v>
+      </c>
+      <c r="F162" t="s">
+        <v>388</v>
+      </c>
+      <c r="G162">
+        <v>85</v>
+      </c>
+      <c r="H162" t="s">
+        <v>385</v>
+      </c>
+      <c r="I162">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="163" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A163" t="s">
+        <v>334</v>
+      </c>
+      <c r="B163" t="s">
+        <v>386</v>
+      </c>
+      <c r="C163">
+        <v>150</v>
+      </c>
+      <c r="D163" t="s">
+        <v>387</v>
+      </c>
+      <c r="E163">
+        <v>120</v>
+      </c>
+      <c r="F163" t="s">
+        <v>388</v>
+      </c>
+      <c r="G163">
+        <v>85</v>
+      </c>
+      <c r="H163" t="s">
+        <v>385</v>
+      </c>
+      <c r="I163">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="164" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A164" t="s">
+        <v>335</v>
+      </c>
+      <c r="B164" t="s">
+        <v>384</v>
+      </c>
+      <c r="C164">
+        <v>120</v>
+      </c>
+      <c r="D164" t="s">
+        <v>386</v>
+      </c>
+      <c r="E164">
+        <v>55</v>
+      </c>
+      <c r="F164" t="s">
+        <v>387</v>
+      </c>
+      <c r="G164">
+        <v>150</v>
+      </c>
+      <c r="H164" t="s">
+        <v>389</v>
+      </c>
+      <c r="I164">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="165" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A165" t="s">
+        <v>336</v>
+      </c>
+      <c r="B165" t="s">
+        <v>384</v>
+      </c>
+      <c r="C165">
+        <v>120</v>
+      </c>
+      <c r="D165" t="s">
+        <v>386</v>
+      </c>
+      <c r="E165">
+        <v>55</v>
+      </c>
+      <c r="F165" t="s">
+        <v>387</v>
+      </c>
+      <c r="G165">
+        <v>150</v>
+      </c>
+      <c r="H165" t="s">
+        <v>389</v>
+      </c>
+      <c r="I165">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="166" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A166" t="s">
+        <v>337</v>
+      </c>
+      <c r="B166" t="s">
+        <v>384</v>
+      </c>
+      <c r="C166">
+        <v>120</v>
+      </c>
+      <c r="D166" t="s">
+        <v>386</v>
+      </c>
+      <c r="E166">
+        <v>55</v>
+      </c>
+      <c r="F166" t="s">
+        <v>387</v>
+      </c>
+      <c r="G166">
+        <v>150</v>
+      </c>
+      <c r="H166" t="s">
+        <v>389</v>
+      </c>
+      <c r="I166">
+        <v>35</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>